<commit_message>
Add phase management + step email nurturing system
- payhome_project_management: Add "フェーズ管理" sheet with Phase 0-3
  detailed tasks, transition checklists, and dashboard phase indicator
- payhome_sales: Add step email design (6 steps with full templates,
  all including unsubscribe URL) and delivery management tracking

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/payhome_project_management.xlsx
+++ b/docs/payhome_project_management.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ダッシュボード" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガントチャート" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="担当別Todo" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todo詳細" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追加Todo受付" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方ガイド" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="フェーズ管理" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガントチャート" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="担当別Todo" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Todo詳細" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追加Todo受付" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方ガイド" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,8 +57,40 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="002E4057"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00E8740C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002E4057"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -119,8 +152,33 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F3F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -142,11 +200,25 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D5D8DC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -201,6 +273,34 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -567,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -580,438 +680,384 @@
     <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>現在のフェーズ：Phase 1 データ基盤構築（進行率 約60%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Phase 1残タスク：GA4実装 / CMS構造化 / リード通知メール / 閲覧履歴UI接続 / CMS永続化</t>
+        </is>
+      </c>
+      <c r="E2" s="24" t="inlineStr">
+        <is>
+          <t>Phase 2移行条件：GA4完了 + CMS構造化完了 + 通知メール稼働 + 掲載3社+ + events 1,000件+</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>ぺいほーむ 事業推進管理シート</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>最終更新: 2026-03-22</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="6"/>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>進捗サマリー</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>カテゴリ</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>全タスク数</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>完了</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>進行中</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>完了率</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>担当</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>事業戦略・収益化</t>
         </is>
       </c>
-      <c r="B6" s="5">
+      <c r="B9" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"収益")+COUNTIF('Todo詳細'!B:B,"戦略")</f>
         <v/>
       </c>
-      <c r="C6" s="5">
+      <c r="C9" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"収益",'Todo詳細'!K:K,"完了")+COUNTIFS('Todo詳細'!B:B,"戦略",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D6" s="5">
+      <c r="D9" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"収益",'Todo詳細'!K:K,"進行中")+COUNTIFS('Todo詳細'!B:B,"戦略",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E6" s="5">
+      <c r="E9" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"収益",'Todo詳細'!K:K,"未着手")+COUNTIFS('Todo詳細'!B:B,"戦略",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F6" s="6">
+      <c r="F9" s="6">
         <f>IF(B6=0,"-",C6/B6)</f>
         <v/>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>経営</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>営業・アライアンス</t>
         </is>
       </c>
-      <c r="B7" s="5">
+      <c r="B10" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"営業")</f>
         <v/>
       </c>
-      <c r="C7" s="5">
+      <c r="C10" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"営業",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D7" s="5">
+      <c r="D10" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"営業",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E7" s="5">
+      <c r="E10" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"営業",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F7" s="6">
+      <c r="F10" s="6">
         <f>IF(B7=0,"-",C7/B7)</f>
         <v/>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>経営/営業</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>掲載品質・リライト</t>
         </is>
       </c>
-      <c r="B8" s="5">
+      <c r="B11" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"品質")</f>
         <v/>
       </c>
-      <c r="C8" s="5">
+      <c r="C11" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"品質",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D8" s="5">
+      <c r="D11" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"品質",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E8" s="5">
+      <c r="E11" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"品質",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F8" s="6">
+      <c r="F11" s="6">
         <f>IF(B8=0,"-",C8/B8)</f>
         <v/>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>コンテンツ</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>集客・マーケティング</t>
         </is>
       </c>
-      <c r="B9" s="5">
+      <c r="B12" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"集客")</f>
         <v/>
       </c>
-      <c r="C9" s="5">
+      <c r="C12" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"集客",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D9" s="5">
+      <c r="D12" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"集客",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E9" s="5">
+      <c r="E12" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"集客",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F9" s="6">
+      <c r="F12" s="6">
         <f>IF(B9=0,"-",C9/B9)</f>
         <v/>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>マーケ</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>オペレーション</t>
         </is>
       </c>
-      <c r="B10" s="5">
+      <c r="B13" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"オペ")</f>
         <v/>
       </c>
-      <c r="C10" s="5">
+      <c r="C13" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"オペ",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D10" s="5">
+      <c r="D13" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"オペ",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E10" s="5">
+      <c r="E13" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"オペ",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F10" s="6">
+      <c r="F13" s="6">
         <f>IF(B10=0,"-",C10/B10)</f>
         <v/>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>CS/経営</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>KPI・計測</t>
         </is>
       </c>
-      <c r="B11" s="5">
+      <c r="B14" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"計測")+COUNTIF('Todo詳細'!B:B,"データ")+COUNTIF('Todo詳細'!B:B,"CV")</f>
         <v/>
       </c>
-      <c r="C11" s="5">
+      <c r="C14" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"計測",'Todo詳細'!K:K,"完了")+COUNTIFS('Todo詳細'!B:B,"データ",'Todo詳細'!K:K,"完了")+COUNTIFS('Todo詳細'!B:B,"CV",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D11" s="5">
+      <c r="D14" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"計測",'Todo詳細'!K:K,"進行中")+COUNTIFS('Todo詳細'!B:B,"データ",'Todo詳細'!K:K,"進行中")+COUNTIFS('Todo詳細'!B:B,"CV",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E11" s="5">
+      <c r="E14" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"計測",'Todo詳細'!K:K,"未着手")+COUNTIFS('Todo詳細'!B:B,"データ",'Todo詳細'!K:K,"未着手")+COUNTIFS('Todo詳細'!B:B,"CV",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F11" s="6">
+      <c r="F14" s="6">
         <f>IF(B11=0,"-",C11/B11)</f>
         <v/>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>PM</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>コンテンツ制作</t>
         </is>
       </c>
-      <c r="B12" s="5">
+      <c r="B15" s="5">
         <f>COUNTIF('Todo詳細'!B:B,"コンテンツ")</f>
         <v/>
       </c>
-      <c r="C12" s="5">
+      <c r="C15" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"コンテンツ",'Todo詳細'!K:K,"完了")</f>
         <v/>
       </c>
-      <c r="D12" s="5">
+      <c r="D15" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"コンテンツ",'Todo詳細'!K:K,"進行中")</f>
         <v/>
       </c>
-      <c r="E12" s="5">
+      <c r="E15" s="5">
         <f>COUNTIFS('Todo詳細'!B:B,"コンテンツ",'Todo詳細'!K:K,"未着手")</f>
         <v/>
       </c>
-      <c r="F12" s="6">
+      <c r="F15" s="6">
         <f>IF(B12=0,"-",C12/B12)</f>
         <v/>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>コンテンツ</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="B13" s="7">
+      <c r="B16" s="7">
         <f>SUM(B6:B12)</f>
         <v/>
       </c>
-      <c r="C13" s="7">
+      <c r="C16" s="7">
         <f>SUM(C6:C12)</f>
         <v/>
       </c>
-      <c r="D13" s="7">
+      <c r="D16" s="7">
         <f>SUM(D6:D12)</f>
         <v/>
       </c>
-      <c r="E13" s="7">
+      <c r="E16" s="7">
         <f>SUM(E6:E12)</f>
         <v/>
       </c>
-      <c r="F13" s="8">
+      <c r="F16" s="8">
         <f>IF(B13=0,"-",C13/B13)</f>
         <v/>
       </c>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>直近マイルストーン</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>マイルストーン</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>目標日</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>状態</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>担当</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>備考</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>営業提案書 完成</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>GA4計測 稼働開始</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>PM/エンジニア</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>初期パートナー1社 獲得</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>経営/営業</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>最重要</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>掲載品質監査 完了</t>
+          <t>営業提案書 完成</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -1021,7 +1067,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>コンテンツ</t>
+          <t>経営</t>
         </is>
       </c>
       <c r="E20" s="5" t="n"/>
@@ -1029,22 +1075,22 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>週次KPIレポート 開始</t>
+          <t>GA4計測 稼働開始</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>PM</t>
+          <t>PM/エンジニア</t>
         </is>
       </c>
       <c r="E21" s="5" t="n"/>
@@ -1052,12 +1098,12 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>パートナー3社 達成</t>
+          <t>初期パートナー1社 獲得</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -1067,36 +1113,111 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>営業</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="n"/>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>最重要</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>掲載品質監査 完了</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>コンテンツ</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>週次KPIレポート 開始</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>パートナー3社 達成</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
           <t>月次売上 発生</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>経営</t>
         </is>
       </c>
-      <c r="E23" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="A2:D2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1104,6 +1225,2034 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E8740C"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>ぺいほーむ フェーズ管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="26" t="inlineStr">
+        <is>
+          <t>フェーズ概要</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>フェーズ</t>
+        </is>
+      </c>
+      <c r="B4" s="27" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>概要</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>開始条件</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>完了条件</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>期間目安</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>事業側の主な作業</t>
+        </is>
+      </c>
+      <c r="H4" s="27" t="inlineStr">
+        <is>
+          <t>開発側の主な作業</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>✅ 完了</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>プラットフォーム基盤構築（62画面・認証・AIチャット基盤）</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>全画面実装完了</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>完了済み</t>
+        </is>
+      </c>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>要件定義・画面設計</t>
+        </is>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>フロントエンド・バックエンド全構築</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>🔧 進行中（約60%）</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>データ基盤構築（行動追跡・チャットログ・お気に入り・GA4）</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Phase 0完了</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>GA4設置完了 + CMS構造化完了 + リード通知メール稼働 + 掲載工務店3社以上 + user_events 1,000件以上</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>1〜2ヶ月</t>
+        </is>
+      </c>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>工務店営業・掲載情報整備・GA4設計・コンテンツ品質改善</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>GA4実装・CMS構造化フォーム・Resendメール接続・閲覧履歴UI接続</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>AI活用開始（推薦・診断・意向抽出・分析ダッシュボード）</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1の完了条件を全て満たす</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>AI推薦精度検証完了 + 月間リード30件以上 + 掲載工務店10社以上 + プロフィール登録率10%以上</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>3〜6ヶ月</t>
+        </is>
+      </c>
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>AI推薦のフィードバック・工務店レポート設計・営業拡大・コンテンツ量産</t>
+        </is>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>user_profiles・比較リスト・AIチャット拡張・推薦ロジック・分析ダッシュボード</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>AI本格稼働・SaaS化（AI住宅コンシェルジュ・AI営業マン・Stripe決済）</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2の完了条件を全て満たす</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>AI住宅コンシェルジュ稼働 + SaaSプラン販売開始 + エリア拡大計画策定</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>6〜12ヶ月</t>
+        </is>
+      </c>
+      <c r="G8" s="28" t="inlineStr">
+        <is>
+          <t>SaaS価格設定・エリア拡大戦略・パートナー拡大</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>AIコンシェルジュ・AI営業マン・Stripe連携・CRM連携</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="26" t="inlineStr">
+        <is>
+          <t>Phase 1：データ基盤構築（詳細）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B11" s="27" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>優先度</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>担当</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
+        <is>
+          <t>事業側Todo</t>
+        </is>
+      </c>
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>開発側Todo</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="inlineStr">
+        <is>
+          <t>完了基準</t>
+        </is>
+      </c>
+      <c r="I11" s="27" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="inlineStr">
+        <is>
+          <t>anonymous_id統一</t>
+        </is>
+      </c>
+      <c r="C12" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>✅ 完了</t>
+        </is>
+      </c>
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="28" t="inlineStr">
+        <is>
+          <t>use-anonymous-id.ts実装済み</t>
+        </is>
+      </c>
+      <c r="H12" s="28" t="inlineStr">
+        <is>
+          <t>LocalStorage生成・保存・送信</t>
+        </is>
+      </c>
+      <c r="I12" s="28" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>P1-02</t>
+        </is>
+      </c>
+      <c r="B13" s="28" t="inlineStr">
+        <is>
+          <t>user_eventsテーブル + API</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>✅ 完了</t>
+        </is>
+      </c>
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F13" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="28" t="inlineStr">
+        <is>
+          <t>POST /api/events/track実装済み</t>
+        </is>
+      </c>
+      <c r="H13" s="28" t="inlineStr">
+        <is>
+          <t>sendBeaconバッチ送信</t>
+        </is>
+      </c>
+      <c r="I13" s="28" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>P1-03</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>chat_sessions / chat_messages保存</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>✅ 完了</t>
+        </is>
+      </c>
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F14" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G14" s="28" t="inlineStr">
+        <is>
+          <t>チャットAPI拡張済み</t>
+        </is>
+      </c>
+      <c r="H14" s="28" t="inlineStr">
+        <is>
+          <t>会話ログがDBに保存される</t>
+        </is>
+      </c>
+      <c r="I14" s="28" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>P1-04</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>リード流入チャネル・直前閲覧付与</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>✅ 完了</t>
+        </is>
+      </c>
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="28" t="inlineStr">
+        <is>
+          <t>inferSourceChannel実装済み</t>
+        </is>
+      </c>
+      <c r="H15" s="28" t="inlineStr">
+        <is>
+          <t>リードにsource_channel, recent_views付与</t>
+        </is>
+      </c>
+      <c r="I15" s="28" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>P1-05</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>お気に入り機能</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>✅ 完了</t>
+        </is>
+      </c>
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G16" s="28" t="inlineStr">
+        <is>
+          <t>FavoriteButton + API実装済み</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="inlineStr">
+        <is>
+          <t>未ログインでも動作・ログイン後マージ</t>
+        </is>
+      </c>
+      <c r="I16" s="28" t="inlineStr">
+        <is>
+          <t>実装済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>P1-06</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>閲覧履歴UI接続</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>⚠️ 部分的</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F17" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>ダッシュボードUIをライブデータに接続</t>
+        </is>
+      </c>
+      <c r="H17" s="28" t="inlineStr">
+        <is>
+          <t>/dashboard/user/historyがリアルデータ表示</t>
+        </is>
+      </c>
+      <c r="I17" s="28" t="inlineStr">
+        <is>
+          <t>モックデータのまま</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>P1-07</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>GA4カスタムイベント設計・実装</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>❌ 未実装</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="inlineStr">
+        <is>
+          <t>計測すべきイベント17種の最終確認・GA4プロパティ設定</t>
+        </is>
+      </c>
+      <c r="G18" s="28" t="inlineStr">
+        <is>
+          <t>gtag()呼び出し追加・カスタムディメンション設定</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="inlineStr">
+        <is>
+          <t>17イベントがGA4で計測できる</t>
+        </is>
+      </c>
+      <c r="I18" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア初タスク</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>P1-08</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>CMS構造化データ項目追加</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>❌ 未実装</t>
+        </is>
+      </c>
+      <c r="E19" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア + 営業</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>工務店に入力してもらう項目の最終決定・工務店への説明</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>CMS編集画面に構造化入力フォーム追加</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="inlineStr">
+        <is>
+          <t>全掲載工務店のdesign_taste/features/suitable_for入力完了</t>
+        </is>
+      </c>
+      <c r="I19" s="28" t="inlineStr">
+        <is>
+          <t>営業側の工務店ヒアリングと連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>P1-09</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Resendリード通知メール</t>
+        </is>
+      </c>
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>❌ 未実装</t>
+        </is>
+      </c>
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="inlineStr">
+        <is>
+          <t>通知先メールアドレスの確認</t>
+        </is>
+      </c>
+      <c r="G20" s="28" t="inlineStr">
+        <is>
+          <t>email.ts → フォーム送信APIへの接続</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="inlineStr">
+        <is>
+          <t>リード発生時に工務店へ即時メール通知</t>
+        </is>
+      </c>
+      <c r="I20" s="28" t="inlineStr">
+        <is>
+          <t>email_notification_spec参照</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>CMS → Supabase永続化</t>
+        </is>
+      </c>
+      <c r="C21" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>❌ 未実装</t>
+        </is>
+      </c>
+      <c r="E21" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G21" s="28" t="inlineStr">
+        <is>
+          <t>TSファイルデータのSupabase移行</t>
+        </is>
+      </c>
+      <c r="H21" s="28" t="inlineStr">
+        <is>
+          <t>CMS編集がDBに保存される</t>
+        </is>
+      </c>
+      <c r="I21" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2の前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>Phase 2：AI活用開始（詳細）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B24" s="27" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>優先度</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>担当</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
+        <is>
+          <t>事業側Todo</t>
+        </is>
+      </c>
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>開発側Todo</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="inlineStr">
+        <is>
+          <t>完了基準</t>
+        </is>
+      </c>
+      <c r="I24" s="27" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>P2-01</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="inlineStr">
+        <is>
+          <t>user_profilesテーブル</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E25" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア + PM</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="inlineStr">
+        <is>
+          <t>プロフィール項目の最終決定（家族構成・予算・希望エリア等）</t>
+        </is>
+      </c>
+      <c r="G25" s="28" t="inlineStr">
+        <is>
+          <t>テーブル作成・API・段階的入力UI</t>
+        </is>
+      </c>
+      <c r="H25" s="28" t="inlineStr">
+        <is>
+          <t>ユーザーがプロフィールを入力・更新できる</t>
+        </is>
+      </c>
+      <c r="I25" s="28" t="inlineStr">
+        <is>
+          <t>段階的プロフィール構築</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="45" customHeight="1">
+      <c r="A26" s="28" t="inlineStr">
+        <is>
+          <t>P2-02</t>
+        </is>
+      </c>
+      <c r="B26" s="28" t="inlineStr">
+        <is>
+          <t>比較リスト機能</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D26" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="28" t="inlineStr">
+        <is>
+          <t>比較テーブル・API・比較UI（横並び表示）</t>
+        </is>
+      </c>
+      <c r="H26" s="28" t="inlineStr">
+        <is>
+          <t>工務店・物件を最大5件まで比較できる</t>
+        </is>
+      </c>
+      <c r="I26" s="28" t="inlineStr">
+        <is>
+          <t>お気に入りと連動</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>P2-03</t>
+        </is>
+      </c>
+      <c r="B27" s="28" t="inlineStr">
+        <is>
+          <t>AIチャット拡張（意向抽出）</t>
+        </is>
+      </c>
+      <c r="C27" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="inlineStr">
+        <is>
+          <t>抽出すべき意向タグの定義（平屋/ZEH/デザイン等）</t>
+        </is>
+      </c>
+      <c r="G27" s="28" t="inlineStr">
+        <is>
+          <t>GPT-4oプロンプト拡張・タグ抽出ロジック</t>
+        </is>
+      </c>
+      <c r="H27" s="28" t="inlineStr">
+        <is>
+          <t>チャット終了時にinterest_tags自動付与</t>
+        </is>
+      </c>
+      <c r="I27" s="28" t="inlineStr">
+        <is>
+          <t>ai_chat_operation_rules参照</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
+      <c r="A28" s="28" t="inlineStr">
+        <is>
+          <t>P2-04</t>
+        </is>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>AIチャット拡張（工務店推薦）</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>推薦ロジックのルール定義（エリア×価格×デザイン）</t>
+        </is>
+      </c>
+      <c r="G28" s="28" t="inlineStr">
+        <is>
+          <t>推薦API・構造化データとのマッチング</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="inlineStr">
+        <is>
+          <t>ユーザーの条件に合う工務店を3社提案</t>
+        </is>
+      </c>
+      <c r="I28" s="28" t="inlineStr">
+        <is>
+          <t>CMS構造化データが前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>P2-05</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>AIチャット拡張（会話要約）</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F29" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G29" s="28" t="inlineStr">
+        <is>
+          <t>GPT-4oによる会話要約の自動生成</t>
+        </is>
+      </c>
+      <c r="H29" s="28" t="inlineStr">
+        <is>
+          <t>chat_sessionsにconversation_summary保存</t>
+        </is>
+      </c>
+      <c r="I29" s="28" t="inlineStr">
+        <is>
+          <t>リード化時に活用</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="45" customHeight="1">
+      <c r="A30" s="28" t="inlineStr">
+        <is>
+          <t>P2-06</t>
+        </is>
+      </c>
+      <c r="B30" s="28" t="inlineStr">
+        <is>
+          <t>意向データ付きリード</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D30" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>工務店に共有するリード情報の最終設計</t>
+        </is>
+      </c>
+      <c r="G30" s="28" t="inlineStr">
+        <is>
+          <t>リード詳細画面に行動履歴・チャット要約・推薦理由を表示</t>
+        </is>
+      </c>
+      <c r="H30" s="28" t="inlineStr">
+        <is>
+          <t>工務店が商談前にユーザーの意向を把握できる</t>
+        </is>
+      </c>
+      <c r="I30" s="28" t="inlineStr">
+        <is>
+          <t>lead_management_rules参照</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>P2-07</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="inlineStr">
+        <is>
+          <t>スコアリング可視化</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D31" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E31" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F31" s="28" t="inlineStr">
+        <is>
+          <t>スコアリングルールの最終調整（重み付け）</t>
+        </is>
+      </c>
+      <c r="G31" s="28" t="inlineStr">
+        <is>
+          <t>行動データからtemperature自動計算・管理画面表示</t>
+        </is>
+      </c>
+      <c r="H31" s="28" t="inlineStr">
+        <is>
+          <t>リード一覧でHot/Warm/Cold表示</t>
+        </is>
+      </c>
+      <c r="I31" s="28" t="inlineStr">
+        <is>
+          <t>lead_management_rules参照</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="45" customHeight="1">
+      <c r="A32" s="28" t="inlineStr">
+        <is>
+          <t>P2-08</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="inlineStr">
+        <is>
+          <t>管理画面分析ダッシュボード</t>
+        </is>
+      </c>
+      <c r="C32" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D32" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E32" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F32" s="28" t="inlineStr">
+        <is>
+          <t>見たいKPIの優先順位決定</t>
+        </is>
+      </c>
+      <c r="G32" s="28" t="inlineStr">
+        <is>
+          <t>チャート・集計API・ダッシュボードUI</t>
+        </is>
+      </c>
+      <c r="H32" s="28" t="inlineStr">
+        <is>
+          <t>チャット・行動・ファネル分析が閲覧できる</t>
+        </is>
+      </c>
+      <c r="I32" s="28" t="inlineStr">
+        <is>
+          <t>GA4データとの連携</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="45" customHeight="1">
+      <c r="A33" s="28" t="inlineStr">
+        <is>
+          <t>P2-09</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="inlineStr">
+        <is>
+          <t>工務店向けレポート基盤</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E33" s="28" t="inlineStr">
+        <is>
+          <t>PM + 営業 + エンジニア</t>
+        </is>
+      </c>
+      <c r="F33" s="28" t="inlineStr">
+        <is>
+          <t>レポートに含める項目・頻度の決定（月次想定）</t>
+        </is>
+      </c>
+      <c r="G33" s="28" t="inlineStr">
+        <is>
+          <t>レポート自動生成・PDF出力・メール送信</t>
+        </is>
+      </c>
+      <c r="H33" s="28" t="inlineStr">
+        <is>
+          <t>工務店に月次でリードレポートが届く</t>
+        </is>
+      </c>
+      <c r="I33" s="28" t="inlineStr">
+        <is>
+          <t>営業価値の核心</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="45" customHeight="1">
+      <c r="A34" s="28" t="inlineStr">
+        <is>
+          <t>P2-10</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="inlineStr">
+        <is>
+          <t>LINE Messaging API連携</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E34" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F34" s="28" t="inlineStr">
+        <is>
+          <t>LINE公式アカウント設定・リッチメニュー設計</t>
+        </is>
+      </c>
+      <c r="G34" s="28" t="inlineStr">
+        <is>
+          <t>友だち追加追跡・プッシュ通知</t>
+        </is>
+      </c>
+      <c r="H34" s="28" t="inlineStr">
+        <is>
+          <t>LINE経由のリード追跡ができる</t>
+        </is>
+      </c>
+      <c r="I34" s="28" t="inlineStr">
+        <is>
+          <t>platform_operation_rules参照</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="26" t="inlineStr">
+        <is>
+          <t>Phase 3：AI本格稼働・SaaS化（詳細）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="27" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B37" s="27" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>優先度</t>
+        </is>
+      </c>
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>担当</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="inlineStr">
+        <is>
+          <t>事業側Todo</t>
+        </is>
+      </c>
+      <c r="G37" s="27" t="inlineStr">
+        <is>
+          <t>開発側Todo</t>
+        </is>
+      </c>
+      <c r="H37" s="27" t="inlineStr">
+        <is>
+          <t>完了基準</t>
+        </is>
+      </c>
+      <c r="I37" s="27" t="inlineStr">
+        <is>
+          <t>備考</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
+      <c r="A38" s="28" t="inlineStr">
+        <is>
+          <t>P3-01</t>
+        </is>
+      </c>
+      <c r="B38" s="28" t="inlineStr">
+        <is>
+          <t>AI住宅コンシェルジュ</t>
+        </is>
+      </c>
+      <c r="C38" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D38" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E38" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F38" s="28" t="inlineStr">
+        <is>
+          <t>コンシェルジュの対話シナリオ設計・品質基準策定</t>
+        </is>
+      </c>
+      <c r="G38" s="28" t="inlineStr">
+        <is>
+          <t>検討フェーズ認識 + 行動文脈 + パーソナライズ対話</t>
+        </is>
+      </c>
+      <c r="H38" s="28" t="inlineStr">
+        <is>
+          <t>ユーザーの検討段階に応じた高度な対話ができる</t>
+        </is>
+      </c>
+      <c r="I38" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2のデータ蓄積が前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="45" customHeight="1">
+      <c r="A39" s="28" t="inlineStr">
+        <is>
+          <t>P3-02</t>
+        </is>
+      </c>
+      <c r="B39" s="28" t="inlineStr">
+        <is>
+          <t>AI営業マン</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E39" s="28" t="inlineStr">
+        <is>
+          <t>PM + 営業 + エンジニア</t>
+        </is>
+      </c>
+      <c r="F39" s="28" t="inlineStr">
+        <is>
+          <t>工務店向け提案支援のユースケース定義</t>
+        </is>
+      </c>
+      <c r="G39" s="28" t="inlineStr">
+        <is>
+          <t>商談支援ダッシュボード・提案自動生成</t>
+        </is>
+      </c>
+      <c r="H39" s="28" t="inlineStr">
+        <is>
+          <t>工務店がAI提案を活用して成約率向上</t>
+        </is>
+      </c>
+      <c r="I39" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2の推薦ロジック改善後</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="45" customHeight="1">
+      <c r="A40" s="28" t="inlineStr">
+        <is>
+          <t>P3-03</t>
+        </is>
+      </c>
+      <c r="B40" s="28" t="inlineStr">
+        <is>
+          <t>商談前要約自動生成</t>
+        </is>
+      </c>
+      <c r="C40" s="28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D40" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E40" s="28" t="inlineStr">
+        <is>
+          <t>エンジニア</t>
+        </is>
+      </c>
+      <c r="F40" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G40" s="28" t="inlineStr">
+        <is>
+          <t>チャット + 行動 + プロフィールの統合要約API</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="inlineStr">
+        <is>
+          <t>工務店が商談前にユーザー要約を確認できる</t>
+        </is>
+      </c>
+      <c r="I40" s="28" t="inlineStr">
+        <is>
+          <t>P2-05, P2-06の延長</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="45" customHeight="1">
+      <c r="A41" s="28" t="inlineStr">
+        <is>
+          <t>P3-04</t>
+        </is>
+      </c>
+      <c r="B41" s="28" t="inlineStr">
+        <is>
+          <t>営業改善SaaS</t>
+        </is>
+      </c>
+      <c r="C41" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E41" s="28" t="inlineStr">
+        <is>
+          <t>経営 + PM</t>
+        </is>
+      </c>
+      <c r="F41" s="28" t="inlineStr">
+        <is>
+          <t>SaaS機能設計・価格設定・ターゲット企業定義</t>
+        </is>
+      </c>
+      <c r="G41" s="28" t="inlineStr">
+        <is>
+          <t>成約パターン分析・最適提案エンジン</t>
+        </is>
+      </c>
+      <c r="H41" s="28" t="inlineStr">
+        <is>
+          <t>SaaSプランとして販売可能な状態</t>
+        </is>
+      </c>
+      <c r="I41" s="28" t="inlineStr">
+        <is>
+          <t>十分な成約データが必要</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="45" customHeight="1">
+      <c r="A42" s="28" t="inlineStr">
+        <is>
+          <t>P3-05</t>
+        </is>
+      </c>
+      <c r="B42" s="28" t="inlineStr">
+        <is>
+          <t>Stripe決済連携</t>
+        </is>
+      </c>
+      <c r="C42" s="28" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E42" s="28" t="inlineStr">
+        <is>
+          <t>経営 + エンジニア</t>
+        </is>
+      </c>
+      <c r="F42" s="28" t="inlineStr">
+        <is>
+          <t>料金プラン最終確定・決済フロー設計</t>
+        </is>
+      </c>
+      <c r="G42" s="28" t="inlineStr">
+        <is>
+          <t>Stripeサブスクリプション・請求管理UI</t>
+        </is>
+      </c>
+      <c r="H42" s="28" t="inlineStr">
+        <is>
+          <t>工務店がオンラインでプラン契約・決済できる</t>
+        </is>
+      </c>
+      <c r="I42" s="28" t="inlineStr">
+        <is>
+          <t>掲載工務店10社以上が前提</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="45" customHeight="1">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t>P3-06</t>
+        </is>
+      </c>
+      <c r="B43" s="28" t="inlineStr">
+        <is>
+          <t>CRM連携</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E43" s="28" t="inlineStr">
+        <is>
+          <t>PM + エンジニア</t>
+        </is>
+      </c>
+      <c r="F43" s="28" t="inlineStr">
+        <is>
+          <t>工務店のCRM利用状況調査・連携先CRM選定</t>
+        </is>
+      </c>
+      <c r="G43" s="28" t="inlineStr">
+        <is>
+          <t>API連携・データ同期</t>
+        </is>
+      </c>
+      <c r="H43" s="28" t="inlineStr">
+        <is>
+          <t>主要CRMにリード情報を自動連携</t>
+        </is>
+      </c>
+      <c r="I43" s="28" t="inlineStr">
+        <is>
+          <t>工務店ニーズ次第</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="45" customHeight="1">
+      <c r="A44" s="28" t="inlineStr">
+        <is>
+          <t>P3-07</t>
+        </is>
+      </c>
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>エリア拡大（九州全域→中国・四国）</t>
+        </is>
+      </c>
+      <c r="C44" s="28" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D44" s="31" t="inlineStr">
+        <is>
+          <t>📋 未着手</t>
+        </is>
+      </c>
+      <c r="E44" s="28" t="inlineStr">
+        <is>
+          <t>経営 + 営業</t>
+        </is>
+      </c>
+      <c r="F44" s="28" t="inlineStr">
+        <is>
+          <t>エリア拡大戦略策定・新規エリア工務店開拓</t>
+        </is>
+      </c>
+      <c r="G44" s="28" t="inlineStr">
+        <is>
+          <t>エリアフィルター拡張・コンテンツ追加</t>
+        </is>
+      </c>
+      <c r="H44" s="28" t="inlineStr">
+        <is>
+          <t>新エリアで掲載工務店5社以上</t>
+        </is>
+      </c>
+      <c r="I44" s="28" t="inlineStr">
+        <is>
+          <t>九州での実績確立後</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="26" t="inlineStr">
+        <is>
+          <t>フェーズ移行条件チェックリスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>移行</t>
+        </is>
+      </c>
+      <c r="B48" s="27" t="inlineStr">
+        <is>
+          <t>チェック項目</t>
+        </is>
+      </c>
+      <c r="C48" s="27" t="inlineStr">
+        <is>
+          <t>現状</t>
+        </is>
+      </c>
+      <c r="D48" s="27" t="inlineStr">
+        <is>
+          <t>達成基準</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr">
+        <is>
+          <t>状態</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1→2</t>
+        </is>
+      </c>
+      <c r="B49" s="28" t="inlineStr">
+        <is>
+          <t>GA4カスタムイベント設置</t>
+        </is>
+      </c>
+      <c r="C49" s="28" t="inlineStr">
+        <is>
+          <t>未実装</t>
+        </is>
+      </c>
+      <c r="D49" s="28" t="inlineStr">
+        <is>
+          <t>17イベントが計測可能</t>
+        </is>
+      </c>
+      <c r="E49" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1→2</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>CMS構造化データ入力</t>
+        </is>
+      </c>
+      <c r="C50" s="28" t="inlineStr">
+        <is>
+          <t>未実装</t>
+        </is>
+      </c>
+      <c r="D50" s="28" t="inlineStr">
+        <is>
+          <t>全掲載工務店の構造化データ入力完了</t>
+        </is>
+      </c>
+      <c r="E50" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1→2</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
+        <is>
+          <t>リード通知メール稼働</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="inlineStr">
+        <is>
+          <t>未実装</t>
+        </is>
+      </c>
+      <c r="D51" s="28" t="inlineStr">
+        <is>
+          <t>Resend経由で即時通知が動作</t>
+        </is>
+      </c>
+      <c r="E51" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1→2</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>掲載工務店数</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>0社（テストデータ）</t>
+        </is>
+      </c>
+      <c r="D52" s="28" t="inlineStr">
+        <is>
+          <t>3社以上の実データ掲載</t>
+        </is>
+      </c>
+      <c r="E52" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1→2</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
+        <is>
+          <t>user_events蓄積量</t>
+        </is>
+      </c>
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>蓄積開始済み</t>
+        </is>
+      </c>
+      <c r="D53" s="28" t="inlineStr">
+        <is>
+          <t>1,000件以上</t>
+        </is>
+      </c>
+      <c r="E53" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="28" t="inlineStr">
+        <is>
+          <t>Phase 1→2</t>
+        </is>
+      </c>
+      <c r="B54" s="28" t="inlineStr">
+        <is>
+          <t>掲載情報品質</t>
+        </is>
+      </c>
+      <c r="C54" s="28" t="inlineStr">
+        <is>
+          <t>未監査</t>
+        </is>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>全工務店ページの文言監査完了</t>
+        </is>
+      </c>
+      <c r="E54" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2→3</t>
+        </is>
+      </c>
+      <c r="B55" s="28" t="inlineStr">
+        <is>
+          <t>AI推薦精度検証</t>
+        </is>
+      </c>
+      <c r="C55" s="28" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>推薦クリック率10%以上</t>
+        </is>
+      </c>
+      <c r="E55" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2→3</t>
+        </is>
+      </c>
+      <c r="B56" s="28" t="inlineStr">
+        <is>
+          <t>月間リード数</t>
+        </is>
+      </c>
+      <c r="C56" s="28" t="inlineStr">
+        <is>
+          <t>0件</t>
+        </is>
+      </c>
+      <c r="D56" s="28" t="inlineStr">
+        <is>
+          <t>30件以上</t>
+        </is>
+      </c>
+      <c r="E56" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2→3</t>
+        </is>
+      </c>
+      <c r="B57" s="28" t="inlineStr">
+        <is>
+          <t>掲載工務店数</t>
+        </is>
+      </c>
+      <c r="C57" s="28" t="inlineStr">
+        <is>
+          <t>0社</t>
+        </is>
+      </c>
+      <c r="D57" s="28" t="inlineStr">
+        <is>
+          <t>10社以上</t>
+        </is>
+      </c>
+      <c r="E57" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2→3</t>
+        </is>
+      </c>
+      <c r="B58" s="28" t="inlineStr">
+        <is>
+          <t>プロフィール登録率</t>
+        </is>
+      </c>
+      <c r="C58" s="28" t="inlineStr">
+        <is>
+          <t>未実装</t>
+        </is>
+      </c>
+      <c r="D58" s="28" t="inlineStr">
+        <is>
+          <t>登録ユーザーの10%以上</t>
+        </is>
+      </c>
+      <c r="E58" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>Phase 2→3</t>
+        </is>
+      </c>
+      <c r="B59" s="28" t="inlineStr">
+        <is>
+          <t>成約データ蓄積</t>
+        </is>
+      </c>
+      <c r="C59" s="28" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="D59" s="28" t="inlineStr">
+        <is>
+          <t>成約50件以上（パターン分析に必要）</t>
+        </is>
+      </c>
+      <c r="E59" s="32" t="inlineStr">
+        <is>
+          <t>❌</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A47:I47"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="A3:I3"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="D12:D21 D25:D34 D38:D44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="無効な値" error="ステータスを選択してください" type="list">
+      <formula1>"✅ 完了,🔧 進行中,⚠️ 部分的,❌ 未実装,📋 未着手"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E49:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"❌,✅"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FF6600"/>
@@ -3506,7 +5655,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E8740C"/>
@@ -4859,14 +7008,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E8740C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4962,6 +7111,11 @@
           <t>追加日</t>
         </is>
       </c>
+      <c r="P1" s="33" t="inlineStr">
+        <is>
+          <t>フェーズ</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -8310,7 +10464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00BBDEFB"/>
@@ -8590,7 +10744,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00E8740C"/>

</xml_diff>

<commit_message>
Fix incorrect task statuses + add ABCD legend and operation rules
- Fix T-11 (SEO article): completed → 未着手 (draft not created)
- Fix T-24 (FAQ): completed → 未着手 (not started, depends on rewrite)
- Fix T-26 (audit): completed → 確認中 (framework exists, detail audit incomplete)
- Fix T-27 (re-hearing): completed → 確認中 (template exists, builder names missing)
- Add ABCD automation criteria legend to Todo詳細 sheet
- Add operation rules (status definitions, completion criteria, review process)
- Add role assignment rules (Claude Code vs human responsibilities per ABCD)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/payhome_project_management.xlsx
+++ b/docs/payhome_project_management.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,8 +89,18 @@
       <color rgb="002E4057"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -177,8 +187,13 @@
         <fgColor rgb="00FADBD8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -214,11 +229,55 @@
         <color rgb="00D5D8DC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -301,6 +360,26 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -713,7 +792,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
@@ -1014,7 +1092,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -7015,14 +7092,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P55"/>
+  <dimension ref="A1:P70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
@@ -7880,11 +7957,13 @@
       </c>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="n">
-        <v>1</v>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
@@ -8803,11 +8882,13 @@
       </c>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="L25" s="5" t="n">
-        <v>1</v>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
@@ -8945,11 +9026,13 @@
       </c>
       <c r="K27" s="9" t="inlineStr">
         <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="L27" s="5" t="n">
-        <v>1</v>
+          <t>確認中</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
       </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
@@ -9016,11 +9099,13 @@
       </c>
       <c r="K28" s="9" t="inlineStr">
         <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="n">
-        <v>1</v>
+          <t>確認中</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
@@ -10283,37 +10368,54 @@
       <c r="N47" s="5" t="n"/>
       <c r="O47" s="5" t="n"/>
     </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr">
-        <is>
-          <t>T-47</t>
-        </is>
-      </c>
-      <c r="B48" s="5" t="n"/>
-      <c r="C48" s="5" t="n"/>
-      <c r="D48" s="5" t="n"/>
-      <c r="E48" s="5" t="n"/>
-      <c r="F48" s="5" t="n"/>
-      <c r="G48" s="5" t="n"/>
-      <c r="H48" s="5" t="n"/>
-      <c r="I48" s="5" t="n"/>
-      <c r="J48" s="5" t="n"/>
-      <c r="K48" s="5" t="n"/>
-      <c r="L48" s="5" t="n"/>
-      <c r="M48" s="5" t="n"/>
-      <c r="N48" s="5" t="n"/>
-      <c r="O48" s="5" t="n"/>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="34" t="inlineStr">
+        <is>
+          <t>自動化判定基準（ABCD）</t>
+        </is>
+      </c>
+      <c r="B48" s="35" t="n"/>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="35" t="n"/>
+      <c r="E48" s="35" t="n"/>
+      <c r="F48" s="35" t="n"/>
+      <c r="G48" s="35" t="n"/>
+      <c r="H48" s="35" t="n"/>
+      <c r="I48" s="35" t="n"/>
+      <c r="J48" s="35" t="n"/>
+      <c r="K48" s="35" t="n"/>
+      <c r="L48" s="35" t="n"/>
+      <c r="M48" s="35" t="n"/>
+      <c r="N48" s="35" t="n"/>
+      <c r="O48" s="35" t="n"/>
+      <c r="P48" s="36" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>T-48</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="n"/>
-      <c r="C49" s="5" t="n"/>
-      <c r="D49" s="5" t="n"/>
-      <c r="E49" s="5" t="n"/>
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
+      <c r="B49" s="27" t="inlineStr">
+        <is>
+          <t>意味</t>
+        </is>
+      </c>
+      <c r="C49" s="27" t="inlineStr">
+        <is>
+          <t>クロードコードの役割</t>
+        </is>
+      </c>
+      <c r="D49" s="27" t="inlineStr">
+        <is>
+          <t>人間の役割</t>
+        </is>
+      </c>
+      <c r="E49" s="27" t="inlineStr">
+        <is>
+          <t>具体例</t>
+        </is>
+      </c>
       <c r="F49" s="5" t="n"/>
       <c r="G49" s="5" t="n"/>
       <c r="H49" s="5" t="n"/>
@@ -10325,16 +10427,32 @@
       <c r="N49" s="5" t="n"/>
       <c r="O49" s="5" t="n"/>
     </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>T-49</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="n"/>
-      <c r="C50" s="5" t="n"/>
-      <c r="D50" s="5" t="n"/>
-      <c r="E50" s="5" t="n"/>
+    <row r="50" ht="60" customHeight="1">
+      <c r="A50" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="inlineStr">
+        <is>
+          <t>ほぼ自動化可能</t>
+        </is>
+      </c>
+      <c r="C50" s="28" t="inlineStr">
+        <is>
+          <t>成果物を完成まで作成。そのまま使えるレベル。</t>
+        </is>
+      </c>
+      <c r="D50" s="28" t="inlineStr">
+        <is>
+          <t>最終確認のみ。内容に問題がなければそのまま採用。</t>
+        </is>
+      </c>
+      <c r="E50" s="28" t="inlineStr">
+        <is>
+          <t>SEOメタデータ一括生成、KPIテンプレート作成、レポート雛形作成</t>
+        </is>
+      </c>
       <c r="F50" s="5" t="n"/>
       <c r="G50" s="5" t="n"/>
       <c r="H50" s="5" t="n"/>
@@ -10346,16 +10464,32 @@
       <c r="N50" s="5" t="n"/>
       <c r="O50" s="5" t="n"/>
     </row>
-    <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>T-50</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="n"/>
-      <c r="C51" s="5" t="n"/>
-      <c r="D51" s="5" t="n"/>
-      <c r="E51" s="5" t="n"/>
+    <row r="51" ht="60" customHeight="1">
+      <c r="A51" s="38" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="inlineStr">
+        <is>
+          <t>AIでたたき台作成、人間レビュー必須</t>
+        </is>
+      </c>
+      <c r="C51" s="28" t="inlineStr">
+        <is>
+          <t>草案・初稿・構成案を作成。ただしそのままは使えない。</t>
+        </is>
+      </c>
+      <c r="D51" s="28" t="inlineStr">
+        <is>
+          <t>内容の正確性確認・表現の調整・事実確認・最終判断。</t>
+        </is>
+      </c>
+      <c r="E51" s="28" t="inlineStr">
+        <is>
+          <t>営業提案書、ペルソナカード、記事下書き、メールテンプレート</t>
+        </is>
+      </c>
       <c r="F51" s="5" t="n"/>
       <c r="G51" s="5" t="n"/>
       <c r="H51" s="5" t="n"/>
@@ -10367,16 +10501,32 @@
       <c r="N51" s="5" t="n"/>
       <c r="O51" s="5" t="n"/>
     </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>T-51</t>
-        </is>
-      </c>
-      <c r="B52" s="5" t="n"/>
-      <c r="C52" s="5" t="n"/>
-      <c r="D52" s="5" t="n"/>
-      <c r="E52" s="5" t="n"/>
+    <row r="52" ht="60" customHeight="1">
+      <c r="A52" s="39" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>AI補助は可能だが人間主導</t>
+        </is>
+      </c>
+      <c r="C52" s="28" t="inlineStr">
+        <is>
+          <t>情報収集・整理・分析の補助。だが判断・実行は人間が行う。</t>
+        </is>
+      </c>
+      <c r="D52" s="28" t="inlineStr">
+        <is>
+          <t>方針決定・実行・調整・外部との調整。AIの出力は参考情報として扱う。</t>
+        </is>
+      </c>
+      <c r="E52" s="28" t="inlineStr">
+        <is>
+          <t>KPI目標設定、コンテンツ企画選定、競合分析の示唆出し</t>
+        </is>
+      </c>
       <c r="F52" s="5" t="n"/>
       <c r="G52" s="5" t="n"/>
       <c r="H52" s="5" t="n"/>
@@ -10388,16 +10538,32 @@
       <c r="N52" s="5" t="n"/>
       <c r="O52" s="5" t="n"/>
     </row>
-    <row r="53">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>T-52</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="n"/>
-      <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
+    <row r="53" ht="60" customHeight="1">
+      <c r="A53" s="40" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B53" s="28" t="inlineStr">
+        <is>
+          <t>人間が実行すべき（自動化非推奨）</t>
+        </is>
+      </c>
+      <c r="C53" s="28" t="inlineStr">
+        <is>
+          <t>関与しない。人間の判断・交渉・関係構築が必須。</t>
+        </is>
+      </c>
+      <c r="D53" s="28" t="inlineStr">
+        <is>
+          <t>全て人間が行う。意思決定・交渉・契約・現場作業・価格決定。</t>
+        </is>
+      </c>
+      <c r="E53" s="28" t="inlineStr">
+        <is>
+          <t>工務店への営業訪問、価格決定、契約締結、撮影・取材</t>
+        </is>
+      </c>
       <c r="F53" s="5" t="n"/>
       <c r="G53" s="5" t="n"/>
       <c r="H53" s="5" t="n"/>
@@ -10451,7 +10617,255 @@
       <c r="N55" s="5" t="n"/>
       <c r="O55" s="5" t="n"/>
     </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="26" t="inlineStr">
+        <is>
+          <t>運用ルール</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="80" customHeight="1">
+      <c r="A57" s="41" t="inlineStr">
+        <is>
+          <t>ステータスの定義</t>
+        </is>
+      </c>
+      <c r="B57" s="28" t="inlineStr">
+        <is>
+          <t>未着手：まだ誰も手をつけていない
+進行中：担当者が作業中
+確認中：成果物はあるが内容の確認・レビューが必要
+完了：成果物が確定し、実務で使える状態
+保留：他のタスクの完了を待つ必要がある</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="41" t="inlineStr">
+        <is>
+          <t>「完了」にする条件</t>
+        </is>
+      </c>
+      <c r="B58" s="28" t="inlineStr">
+        <is>
+          <t>● 成果物が存在する（ファイル・シート・ドキュメント等）
+● 内容が実データに基づいている（テンプレートやプレースホルダーのままではない）
+● 担当者が確認済み
+● そのまま実務で使える状態</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="80" customHeight="1">
+      <c r="A59" s="41" t="inlineStr">
+        <is>
+          <t>クロードコードが作った成果物の扱い</t>
+        </is>
+      </c>
+      <c r="B59" s="28" t="inlineStr">
+        <is>
+          <t>● A判定のタスク：最終確認後、そのまま「完了」にしてOK
+● B判定のタスク：草案作成時点では「確認中」。人間がレビュー・修正後に「完了」
+● C/D判定のタスク：AIの出力があっても「確認中」止まり。人間が実行・判断して初めて「完了」</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="41" t="inlineStr">
+        <is>
+          <t>週次レビューのやり方</t>
+        </is>
+      </c>
+      <c r="B60" s="28" t="inlineStr">
+        <is>
+          <t>1. ダッシュボードで全体進捗を確認
+2. フェーズ管理シートで現在フェーズの残タスクを確認
+3. ガントチャートで期限遅れを確認
+4. 担当別Todoで各メンバーのタスクを確認
+5. 「確認中」ステータスのタスクを優先的にレビュー</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="80" customHeight="1">
+      <c r="A61" s="41" t="inlineStr">
+        <is>
+          <t>フェーズ移行の判断</t>
+        </is>
+      </c>
+      <c r="B61" s="28" t="inlineStr">
+        <is>
+          <t>フェーズ管理シートの「フェーズ移行条件チェックリスト」を全員で確認。
+全項目が✅になったら次フェーズに移行。
+移行時には次フェーズのTodoを「未着手」から「進行中」に更新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="80" customHeight="1">
+      <c r="A62" s="41" t="inlineStr">
+        <is>
+          <t>新規タスクの追加方法</t>
+        </is>
+      </c>
+      <c r="B62" s="28" t="inlineStr">
+        <is>
+          <t>「追加Todo受付」シートに記入。
+週次レビューで優先度を判断し、Todo詳細に移動。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="26" t="inlineStr">
+        <is>
+          <t>担当分担ルール</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="27" t="inlineStr">
+        <is>
+          <t>判定</t>
+        </is>
+      </c>
+      <c r="B66" s="27" t="inlineStr">
+        <is>
+          <t>クロードコードがやること</t>
+        </is>
+      </c>
+      <c r="C66" s="27" t="inlineStr">
+        <is>
+          <t>終わった後のステータス</t>
+        </is>
+      </c>
+      <c r="D66" s="27" t="inlineStr">
+        <is>
+          <t>人間がやること</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr">
+        <is>
+          <t>完了後のステータス</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="45" customHeight="1">
+      <c r="A67" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B67" s="28" t="inlineStr">
+        <is>
+          <t>成果物を完成まで作成</t>
+        </is>
+      </c>
+      <c r="C67" s="28" t="inlineStr">
+        <is>
+          <t>→ 確認中</t>
+        </is>
+      </c>
+      <c r="D67" s="28" t="inlineStr">
+        <is>
+          <t>内容を確認して問題なければ承認</t>
+        </is>
+      </c>
+      <c r="E67" s="28" t="inlineStr">
+        <is>
+          <t>→ 完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="45" customHeight="1">
+      <c r="A68" s="38" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B68" s="28" t="inlineStr">
+        <is>
+          <t>草案・初稿・構成案を作成</t>
+        </is>
+      </c>
+      <c r="C68" s="28" t="inlineStr">
+        <is>
+          <t>→ 確認中</t>
+        </is>
+      </c>
+      <c r="D68" s="28" t="inlineStr">
+        <is>
+          <t>内容をレビュー・修正・事実確認して確定</t>
+        </is>
+      </c>
+      <c r="E68" s="28" t="inlineStr">
+        <is>
+          <t>→ 完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="45" customHeight="1">
+      <c r="A69" s="39" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B69" s="28" t="inlineStr">
+        <is>
+          <t>情報収集・分析・整理の補助</t>
+        </is>
+      </c>
+      <c r="C69" s="28" t="inlineStr">
+        <is>
+          <t>→ 確認中</t>
+        </is>
+      </c>
+      <c r="D69" s="28" t="inlineStr">
+        <is>
+          <t>判断・実行・外部調整を行う</t>
+        </is>
+      </c>
+      <c r="E69" s="28" t="inlineStr">
+        <is>
+          <t>→ 完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="45" customHeight="1">
+      <c r="A70" s="40" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B70" s="28" t="inlineStr">
+        <is>
+          <t>関与しない</t>
+        </is>
+      </c>
+      <c r="C70" s="28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="28" t="inlineStr">
+        <is>
+          <t>全て人間が実行（交渉・契約・撮影等）</t>
+        </is>
+      </c>
+      <c r="E70" s="28" t="inlineStr">
+        <is>
+          <t>→ 完了</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B59:P59"/>
+    <mergeCell ref="A56:P56"/>
+    <mergeCell ref="B60:P60"/>
+    <mergeCell ref="B61:P61"/>
+    <mergeCell ref="B57:P57"/>
+    <mergeCell ref="A48:P48"/>
+    <mergeCell ref="B58:P58"/>
+    <mergeCell ref="A65:P65"/>
+    <mergeCell ref="B62:P62"/>
+  </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="K2:K60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"未着手,進行中,確認中,完了,保留"</formula1>

</xml_diff>

<commit_message>
Update project management: add human tasks, fix formulas, sync all sheets
- Fix dashboard F column formulas (wrong row references)
- Add 10 new human tasks (T-45 to T-54): bank partnership, real estate alliance,
  exhibition, insurance, subsidies, Instagram, survey, CS setup, photos, competitor analysis
- Link dashboard summary to Todo詳細 via COUNTIF (auto-updates)
- Link milestone status to Todo詳細 via VLOOKUP (auto-updates)
- Add 5 new milestones (bank, survey, CS, photos, competitor)
- Sync ガントチャート and 担当別Todo with new tasks

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/payhome_project_management.xlsx
+++ b/docs/payhome_project_management.xlsx
@@ -193,7 +193,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -273,11 +273,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D5D8DC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D5D8DC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D5D8DC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -380,6 +424,25 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -746,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -843,23 +906,23 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"収益")+COUNTIF('Todo詳細'!B:B,"戦略")</f>
+        <f>COUNTIF(Todo詳細!B:B,"収益")+COUNTIF(Todo詳細!B:B,"戦略")</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"収益",'Todo詳細'!K:K,"完了")+COUNTIFS('Todo詳細'!B:B,"戦略",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"収益",Todo詳細!K:K,"完了")+COUNTIFS(Todo詳細!B:B,"戦略",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"収益",'Todo詳細'!K:K,"進行中")+COUNTIFS('Todo詳細'!B:B,"戦略",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"収益",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"収益",Todo詳細!K:K,"確認中")+COUNTIFS(Todo詳細!B:B,"戦略",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"戦略",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E9" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"収益",'Todo詳細'!K:K,"未着手")+COUNTIFS('Todo詳細'!B:B,"戦略",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"収益",Todo詳細!K:K,"未着手")+COUNTIFS(Todo詳細!B:B,"戦略",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F9" s="6">
-        <f>IF(B6=0,"-",C6/B6)</f>
+        <f>IF(B9=0,"-",C9/B9)</f>
         <v/>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -875,23 +938,23 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"営業")</f>
+        <f>COUNTIF(Todo詳細!B:B,"営業")</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"営業",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"営業",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"営業",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"営業",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"営業",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E10" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"営業",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"営業",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F10" s="6">
-        <f>IF(B7=0,"-",C7/B7)</f>
+        <f>IF(B10=0,"-",C10/B10)</f>
         <v/>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -907,23 +970,23 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"品質")</f>
+        <f>COUNTIF(Todo詳細!B:B,"品質")</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"品質",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"品質",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"品質",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"品質",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"品質",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E11" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"品質",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"品質",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F11" s="6">
-        <f>IF(B8=0,"-",C8/B8)</f>
+        <f>IF(B11=0,"-",C11/B11)</f>
         <v/>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -939,23 +1002,23 @@
         </is>
       </c>
       <c r="B12" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"集客")</f>
+        <f>COUNTIF(Todo詳細!B:B,"集客")</f>
         <v/>
       </c>
       <c r="C12" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"集客",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"集客",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D12" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"集客",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"集客",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"集客",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E12" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"集客",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"集客",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F12" s="6">
-        <f>IF(B9=0,"-",C9/B9)</f>
+        <f>IF(B12=0,"-",C12/B12)</f>
         <v/>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -971,23 +1034,23 @@
         </is>
       </c>
       <c r="B13" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"オペ")</f>
+        <f>COUNTIF(Todo詳細!B:B,"オペ")</f>
         <v/>
       </c>
       <c r="C13" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"オペ",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"オペ",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D13" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"オペ",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"オペ",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"オペ",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E13" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"オペ",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"オペ",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F13" s="6">
-        <f>IF(B10=0,"-",C10/B10)</f>
+        <f>IF(B13=0,"-",C13/B13)</f>
         <v/>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -1003,23 +1066,23 @@
         </is>
       </c>
       <c r="B14" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"計測")+COUNTIF('Todo詳細'!B:B,"データ")+COUNTIF('Todo詳細'!B:B,"CV")</f>
+        <f>COUNTIF(Todo詳細!B:B,"計測")+COUNTIF(Todo詳細!B:B,"データ")</f>
         <v/>
       </c>
       <c r="C14" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"計測",'Todo詳細'!K:K,"完了")+COUNTIFS('Todo詳細'!B:B,"データ",'Todo詳細'!K:K,"完了")+COUNTIFS('Todo詳細'!B:B,"CV",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"計測",Todo詳細!K:K,"完了")+COUNTIFS(Todo詳細!B:B,"データ",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D14" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"計測",'Todo詳細'!K:K,"進行中")+COUNTIFS('Todo詳細'!B:B,"データ",'Todo詳細'!K:K,"進行中")+COUNTIFS('Todo詳細'!B:B,"CV",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"計測",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"計測",Todo詳細!K:K,"確認中")+COUNTIFS(Todo詳細!B:B,"データ",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"データ",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E14" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"計測",'Todo詳細'!K:K,"未着手")+COUNTIFS('Todo詳細'!B:B,"データ",'Todo詳細'!K:K,"未着手")+COUNTIFS('Todo詳細'!B:B,"CV",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"計測",Todo詳細!K:K,"未着手")+COUNTIFS(Todo詳細!B:B,"データ",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F14" s="6">
-        <f>IF(B11=0,"-",C11/B11)</f>
+        <f>IF(B14=0,"-",C14/B14)</f>
         <v/>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1035,23 +1098,23 @@
         </is>
       </c>
       <c r="B15" s="5">
-        <f>COUNTIF('Todo詳細'!B:B,"コンテンツ")</f>
+        <f>COUNTIF(Todo詳細!B:B,"コンテンツ")+COUNTIF(Todo詳細!B:B,"CV")</f>
         <v/>
       </c>
       <c r="C15" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"コンテンツ",'Todo詳細'!K:K,"完了")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"コンテンツ",Todo詳細!K:K,"完了")+COUNTIFS(Todo詳細!B:B,"CV",Todo詳細!K:K,"完了")</f>
         <v/>
       </c>
       <c r="D15" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"コンテンツ",'Todo詳細'!K:K,"進行中")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"コンテンツ",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"コンテンツ",Todo詳細!K:K,"確認中")+COUNTIFS(Todo詳細!B:B,"CV",Todo詳細!K:K,"進行中")+COUNTIFS(Todo詳細!B:B,"CV",Todo詳細!K:K,"確認中")</f>
         <v/>
       </c>
       <c r="E15" s="5">
-        <f>COUNTIFS('Todo詳細'!B:B,"コンテンツ",'Todo詳細'!K:K,"未着手")</f>
+        <f>COUNTIFS(Todo詳細!B:B,"コンテンツ",Todo詳細!K:K,"未着手")+COUNTIFS(Todo詳細!B:B,"CV",Todo詳細!K:K,"未着手")</f>
         <v/>
       </c>
       <c r="F15" s="6">
-        <f>IF(B12=0,"-",C12/B12)</f>
+        <f>IF(B15=0,"-",C15/B15)</f>
         <v/>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1067,23 +1130,23 @@
         </is>
       </c>
       <c r="B16" s="7">
-        <f>SUM(B6:B12)</f>
+        <f>SUM(B9:B15)</f>
         <v/>
       </c>
       <c r="C16" s="7">
-        <f>SUM(C6:C12)</f>
+        <f>SUM(C9:C15)</f>
         <v/>
       </c>
       <c r="D16" s="7">
-        <f>SUM(D6:D12)</f>
+        <f>SUM(D9:D15)</f>
         <v/>
       </c>
       <c r="E16" s="7">
-        <f>SUM(E6:E12)</f>
+        <f>SUM(E9:E15)</f>
         <v/>
       </c>
       <c r="F16" s="8">
-        <f>IF(B13=0,"-",C13/B13)</f>
+        <f>IF(B16=0,"-",C16/B16)</f>
         <v/>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -1137,10 +1200,9 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
+      <c r="C20" s="9">
+        <f>VLOOKUP("T-07",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
@@ -1160,10 +1222,9 @@
           <t>2026-04-01</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
+      <c r="C21" s="5">
+        <f>VLOOKUP("T-09",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
@@ -1183,10 +1244,9 @@
           <t>2026-04-15</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>未着手</t>
-        </is>
+      <c r="C22" s="5">
+        <f>VLOOKUP("T-36",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
@@ -1210,10 +1270,9 @@
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
+      <c r="C23" s="9">
+        <f>VLOOKUP("T-26",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
@@ -1233,10 +1292,9 @@
           <t>2026-04-07</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
+      <c r="C24" s="9">
+        <f>VLOOKUP("T-38",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
@@ -1290,6 +1348,136 @@
         </is>
       </c>
       <c r="E26" s="5" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>銀行提携 交渉開始</t>
+        </is>
+      </c>
+      <c r="B27" s="42" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C27" s="42">
+        <f>VLOOKUP("T-45",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="E27" s="42" t="inlineStr">
+        <is>
+          <t>住宅ローン特別金利</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="42" t="inlineStr">
+        <is>
+          <t>視聴者アンケート 完了</t>
+        </is>
+      </c>
+      <c r="B28" s="42" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="C28" s="42">
+        <f>VLOOKUP("T-51",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D28" s="42" t="inlineStr">
+        <is>
+          <t>経営/マーケ</t>
+        </is>
+      </c>
+      <c r="E28" s="42" t="inlineStr">
+        <is>
+          <t>ペルソナ更新に使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="42" t="inlineStr">
+        <is>
+          <t>CS体制 構築完了</t>
+        </is>
+      </c>
+      <c r="B29" s="42" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C29" s="42">
+        <f>VLOOKUP("T-52",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>経営/CS</t>
+        </is>
+      </c>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>反響対応開始前に必須</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="42" t="inlineStr">
+        <is>
+          <t>施工事例写真 3社分確保</t>
+        </is>
+      </c>
+      <c r="B30" s="42" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C30" s="42">
+        <f>VLOOKUP("T-53",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D30" s="42" t="inlineStr">
+        <is>
+          <t>コンテンツ/営業</t>
+        </is>
+      </c>
+      <c r="E30" s="42" t="inlineStr">
+        <is>
+          <t>掲載品質に直結</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="42" t="inlineStr">
+        <is>
+          <t>競合分析 完了</t>
+        </is>
+      </c>
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C31" s="42">
+        <f>VLOOKUP("T-54",Todo詳細!A:K,11,FALSE)</f>
+        <v/>
+      </c>
+      <c r="D31" s="42" t="inlineStr">
+        <is>
+          <t>経営/PM</t>
+        </is>
+      </c>
+      <c r="E31" s="42" t="inlineStr">
+        <is>
+          <t>営業提案の差別化根拠</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3336,7 +3524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:V54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5716,6 +5904,326 @@
       <c r="S44" s="13" t="n"/>
       <c r="T44" s="12" t="n"/>
       <c r="U44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="43" t="inlineStr">
+        <is>
+          <t>T-45</t>
+        </is>
+      </c>
+      <c r="B45" s="43" t="inlineStr">
+        <is>
+          <t>銀行への提案（ぺいほーむ特別金利）</t>
+        </is>
+      </c>
+      <c r="C45" s="43" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="D45" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E45" s="43" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F45" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="43" t="inlineStr">
+        <is>
+          <t>T-46</t>
+        </is>
+      </c>
+      <c r="B46" s="43" t="inlineStr">
+        <is>
+          <t>不動産会社との提携交渉</t>
+        </is>
+      </c>
+      <c r="C46" s="43" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="E46" s="43" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="F46" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="43" t="inlineStr">
+        <is>
+          <t>T-47</t>
+        </is>
+      </c>
+      <c r="B47" s="43" t="inlineStr">
+        <is>
+          <t>住宅展示場・イベント出展交渉</t>
+        </is>
+      </c>
+      <c r="C47" s="43" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="D47" s="43" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="E47" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F47" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="43" t="inlineStr">
+        <is>
+          <t>T-48</t>
+        </is>
+      </c>
+      <c r="B48" s="43" t="inlineStr">
+        <is>
+          <t>火災保険・引越し業者アライアンス</t>
+        </is>
+      </c>
+      <c r="C48" s="43" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="E48" s="43" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F48" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="43" t="inlineStr">
+        <is>
+          <t>T-49</t>
+        </is>
+      </c>
+      <c r="B49" s="43" t="inlineStr">
+        <is>
+          <t>補助金・助成金情報の定期更新</t>
+        </is>
+      </c>
+      <c r="C49" s="43" t="inlineStr">
+        <is>
+          <t>コンテンツ</t>
+        </is>
+      </c>
+      <c r="D49" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E49" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F49" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="43" t="inlineStr">
+        <is>
+          <t>T-50</t>
+        </is>
+      </c>
+      <c r="B50" s="43" t="inlineStr">
+        <is>
+          <t>Instagram運用開始</t>
+        </is>
+      </c>
+      <c r="C50" s="43" t="inlineStr">
+        <is>
+          <t>マーケ</t>
+        </is>
+      </c>
+      <c r="D50" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="E50" s="43" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="F50" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="43" t="inlineStr">
+        <is>
+          <t>T-51</t>
+        </is>
+      </c>
+      <c r="B51" s="43" t="inlineStr">
+        <is>
+          <t>既存YouTube視聴者アンケート実施</t>
+        </is>
+      </c>
+      <c r="C51" s="43" t="inlineStr">
+        <is>
+          <t>経営/マーケ</t>
+        </is>
+      </c>
+      <c r="D51" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E51" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="F51" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="43" t="inlineStr">
+        <is>
+          <t>T-52</t>
+        </is>
+      </c>
+      <c r="B52" s="43" t="inlineStr">
+        <is>
+          <t>カスタマーサポート体制構築</t>
+        </is>
+      </c>
+      <c r="C52" s="43" t="inlineStr">
+        <is>
+          <t>経営/CS</t>
+        </is>
+      </c>
+      <c r="D52" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="E52" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F52" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="43" t="inlineStr">
+        <is>
+          <t>T-53</t>
+        </is>
+      </c>
+      <c r="B53" s="43" t="inlineStr">
+        <is>
+          <t>掲載工務店の施工事例写真収集</t>
+        </is>
+      </c>
+      <c r="C53" s="43" t="inlineStr">
+        <is>
+          <t>コンテンツ/営業</t>
+        </is>
+      </c>
+      <c r="D53" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="E53" s="43" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F53" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="43" t="inlineStr">
+        <is>
+          <t>T-54</t>
+        </is>
+      </c>
+      <c r="B54" s="43" t="inlineStr">
+        <is>
+          <t>競合分析レポート作成</t>
+        </is>
+      </c>
+      <c r="C54" s="43" t="inlineStr">
+        <is>
+          <t>経営/PM</t>
+        </is>
+      </c>
+      <c r="D54" s="43" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="E54" s="43" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F54" s="43" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5801,393 +6309,417 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="n"/>
-      <c r="B2" s="16" t="n"/>
-      <c r="C2" s="16" t="n"/>
-      <c r="D2" s="16" t="n"/>
-      <c r="E2" s="16" t="n"/>
-      <c r="F2" s="16" t="n"/>
+      <c r="A2" s="44" t="inlineStr">
+        <is>
+          <t>T-45</t>
+        </is>
+      </c>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="C2" s="44" t="inlineStr">
+        <is>
+          <t>銀行への提案（ぺいほーむ特別金利）</t>
+        </is>
+      </c>
+      <c r="D2" s="44" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E2" s="44" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="F2" s="44" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
       <c r="G2" s="16" t="n"/>
       <c r="H2" s="16" t="n"/>
       <c r="I2" s="16" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>T-06</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>エレベーターピッチ作成</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>戦略</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>03/28</t>
-        </is>
-      </c>
-      <c r="F3" s="18" t="inlineStr">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>T-46</t>
+        </is>
+      </c>
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="C3" s="46" t="inlineStr">
+        <is>
+          <t>不動産会社との提携交渉</t>
+        </is>
+      </c>
+      <c r="D3" s="46" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E3" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="F3" s="47" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>AIで草案3パターン生成→選定</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="45" t="inlineStr">
+        <is>
+          <t>T-47</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>住宅展示場・イベント出展交渉</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E4" s="46" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F4" s="47" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>AIで構成案作成→レビュー</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="45" t="inlineStr">
+        <is>
+          <t>T-48</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>火災保険・引越し業者アライアンス</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="F5" s="47" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>競合調査→3プラン価格決定</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="45" t="inlineStr">
+        <is>
+          <t>T-49</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>コンテンツ</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>補助金・助成金情報の定期更新</t>
+        </is>
+      </c>
+      <c r="D6" s="46" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="F6" s="47" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>完了</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>AIで草案3パターン生成→選定</t>
-        </is>
-      </c>
-      <c r="I3" s="5" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>T-07</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>営業提案書 初稿</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>営業</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>04/04</t>
-        </is>
-      </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>AIでフロー草案→調整</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="45" t="inlineStr">
+        <is>
+          <t>T-50</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>マーケ</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>Instagram運用開始</t>
+        </is>
+      </c>
+      <c r="D7" s="46" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E7" s="46" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="F7" s="47" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>AIでフロー草案→確定</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="45" t="inlineStr">
+        <is>
+          <t>T-51</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>経営/マーケ</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>既存YouTube視聴者アンケート実施</t>
+        </is>
+      </c>
+      <c r="D8" s="46" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>AIで構成案作成→レビュー</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>T-35</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>料金プラン確定</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>収益</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>04/07</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="F8" s="47" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>アポ取得→提案書持参→交渉</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="45" t="inlineStr">
+        <is>
+          <t>T-52</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>経営/CS</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>カスタマーサポート体制構築</t>
+        </is>
+      </c>
+      <c r="D9" s="46" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="F9" s="47" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>競合調査→3プラン価格決定</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>T-17</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>営業フロー設計</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>営業</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>04/07</t>
-        </is>
-      </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>T-19の結果→契約締結</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>最重要</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="45" t="inlineStr">
+        <is>
+          <t>T-53</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>コンテンツ/営業</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>掲載工務店の施工事例写真収集</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>AIでフロー草案→調整</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>T-32</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>問い合わせ対応フロー</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>オペ</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>04/04</t>
-        </is>
-      </c>
-      <c r="F7" s="18" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>完了</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>AIでフロー草案→確定</t>
-        </is>
-      </c>
-      <c r="I7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>T-19</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>既存取材先への提案</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>営業</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>04/18</t>
-        </is>
-      </c>
-      <c r="F8" s="18" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G8" s="16" t="inlineStr">
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F10" s="47" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>アポ取得→提案書持参→交渉</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>T-36</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>初期パートナー1社獲得</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>収益</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>04/25</t>
-        </is>
-      </c>
-      <c r="F9" s="18" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>未着手</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>T-19の結果→契約締結</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>最重要</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>T-40</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>四半期マイルストーン</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>戦略</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>04/07</t>
-        </is>
-      </c>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>高</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="inlineStr">
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Q2/Q3/Q4目標値設定</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="45" t="inlineStr">
+        <is>
+          <t>T-54</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>経営/PM</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>競合分析レポート作成</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="F11" s="47" t="inlineStr">
         <is>
           <t>未着手</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Q2/Q3/Q4目標値設定</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>経営</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>T-08</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>料金プラン確定</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>収益</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>04/07</t>
-        </is>
-      </c>
-      <c r="F11" s="18" t="inlineStr">
-        <is>
-          <t>高</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
@@ -7092,7 +7624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P70"/>
+  <dimension ref="A1:P79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10327,46 +10859,168 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="A46" s="46" t="inlineStr">
         <is>
           <t>T-45</t>
         </is>
       </c>
-      <c r="B46" s="5" t="n"/>
-      <c r="C46" s="5" t="n"/>
-      <c r="D46" s="5" t="n"/>
-      <c r="E46" s="5" t="n"/>
-      <c r="F46" s="5" t="n"/>
-      <c r="G46" s="5" t="n"/>
-      <c r="H46" s="5" t="n"/>
-      <c r="I46" s="5" t="n"/>
-      <c r="J46" s="5" t="n"/>
-      <c r="K46" s="5" t="n"/>
-      <c r="L46" s="5" t="n"/>
-      <c r="M46" s="5" t="n"/>
-      <c r="N46" s="5" t="n"/>
-      <c r="O46" s="5" t="n"/>
+      <c r="B46" s="46" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="C46" s="46" t="inlineStr">
+        <is>
+          <t>銀行への提案（ぺいほーむ特別金利）</t>
+        </is>
+      </c>
+      <c r="D46" s="46" t="inlineStr">
+        <is>
+          <t>住宅ローン連携で差別化</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="inlineStr">
+        <is>
+          <t>地銀・信金にぺいほーむ経由の住宅ローン特別金利を提案</t>
+        </is>
+      </c>
+      <c r="F46" s="46" t="inlineStr">
+        <is>
+          <t>提携契約書/特別金利プラン</t>
+        </is>
+      </c>
+      <c r="G46" s="46" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="H46" s="46" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="I46" s="46" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="J46" s="46" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="K46" s="46" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L46" s="46" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M46" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N46" s="46" t="inlineStr">
+        <is>
+          <t>鹿児島銀行/南日本銀行が候補</t>
+        </is>
+      </c>
+      <c r="O46" s="46" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P46" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr">
+      <c r="A47" s="46" t="inlineStr">
         <is>
           <t>T-46</t>
         </is>
       </c>
-      <c r="B47" s="5" t="n"/>
-      <c r="C47" s="5" t="n"/>
-      <c r="D47" s="5" t="n"/>
-      <c r="E47" s="5" t="n"/>
-      <c r="F47" s="5" t="n"/>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="5" t="n"/>
-      <c r="I47" s="5" t="n"/>
-      <c r="J47" s="5" t="n"/>
-      <c r="K47" s="5" t="n"/>
-      <c r="L47" s="5" t="n"/>
-      <c r="M47" s="5" t="n"/>
-      <c r="N47" s="5" t="n"/>
-      <c r="O47" s="5" t="n"/>
+      <c r="B47" s="46" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="C47" s="46" t="inlineStr">
+        <is>
+          <t>不動産会社との提携交渉</t>
+        </is>
+      </c>
+      <c r="D47" s="46" t="inlineStr">
+        <is>
+          <t>土地探しからワンストップ支援</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="inlineStr">
+        <is>
+          <t>鹿児島・福岡の不動産会社に土地情報連携を提案</t>
+        </is>
+      </c>
+      <c r="F47" s="46" t="inlineStr">
+        <is>
+          <t>提携契約/土地情報連携フロー</t>
+        </is>
+      </c>
+      <c r="G47" s="46" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="H47" s="46" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="I47" s="46" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="J47" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="K47" s="46" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L47" s="46" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M47" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N47" s="46" t="inlineStr">
+        <is>
+          <t>平屋向き土地（50坪以上）</t>
+        </is>
+      </c>
+      <c r="O47" s="46" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P47" s="48" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="34" t="inlineStr">
@@ -10639,6 +11293,20 @@
 保留：他のタスクの完了を待つ必要がある</t>
         </is>
       </c>
+      <c r="C57" s="49" t="n"/>
+      <c r="D57" s="49" t="n"/>
+      <c r="E57" s="49" t="n"/>
+      <c r="F57" s="49" t="n"/>
+      <c r="G57" s="49" t="n"/>
+      <c r="H57" s="49" t="n"/>
+      <c r="I57" s="49" t="n"/>
+      <c r="J57" s="49" t="n"/>
+      <c r="K57" s="49" t="n"/>
+      <c r="L57" s="49" t="n"/>
+      <c r="M57" s="49" t="n"/>
+      <c r="N57" s="49" t="n"/>
+      <c r="O57" s="49" t="n"/>
+      <c r="P57" s="50" t="n"/>
     </row>
     <row r="58" ht="80" customHeight="1">
       <c r="A58" s="41" t="inlineStr">
@@ -10654,6 +11322,20 @@
 ● そのまま実務で使える状態</t>
         </is>
       </c>
+      <c r="C58" s="49" t="n"/>
+      <c r="D58" s="49" t="n"/>
+      <c r="E58" s="49" t="n"/>
+      <c r="F58" s="49" t="n"/>
+      <c r="G58" s="49" t="n"/>
+      <c r="H58" s="49" t="n"/>
+      <c r="I58" s="49" t="n"/>
+      <c r="J58" s="49" t="n"/>
+      <c r="K58" s="49" t="n"/>
+      <c r="L58" s="49" t="n"/>
+      <c r="M58" s="49" t="n"/>
+      <c r="N58" s="49" t="n"/>
+      <c r="O58" s="49" t="n"/>
+      <c r="P58" s="50" t="n"/>
     </row>
     <row r="59" ht="80" customHeight="1">
       <c r="A59" s="41" t="inlineStr">
@@ -10668,6 +11350,20 @@
 ● C/D判定のタスク：AIの出力があっても「確認中」止まり。人間が実行・判断して初めて「完了」</t>
         </is>
       </c>
+      <c r="C59" s="49" t="n"/>
+      <c r="D59" s="49" t="n"/>
+      <c r="E59" s="49" t="n"/>
+      <c r="F59" s="49" t="n"/>
+      <c r="G59" s="49" t="n"/>
+      <c r="H59" s="49" t="n"/>
+      <c r="I59" s="49" t="n"/>
+      <c r="J59" s="49" t="n"/>
+      <c r="K59" s="49" t="n"/>
+      <c r="L59" s="49" t="n"/>
+      <c r="M59" s="49" t="n"/>
+      <c r="N59" s="49" t="n"/>
+      <c r="O59" s="49" t="n"/>
+      <c r="P59" s="50" t="n"/>
     </row>
     <row r="60" ht="80" customHeight="1">
       <c r="A60" s="41" t="inlineStr">
@@ -10684,6 +11380,20 @@
 5. 「確認中」ステータスのタスクを優先的にレビュー</t>
         </is>
       </c>
+      <c r="C60" s="49" t="n"/>
+      <c r="D60" s="49" t="n"/>
+      <c r="E60" s="49" t="n"/>
+      <c r="F60" s="49" t="n"/>
+      <c r="G60" s="49" t="n"/>
+      <c r="H60" s="49" t="n"/>
+      <c r="I60" s="49" t="n"/>
+      <c r="J60" s="49" t="n"/>
+      <c r="K60" s="49" t="n"/>
+      <c r="L60" s="49" t="n"/>
+      <c r="M60" s="49" t="n"/>
+      <c r="N60" s="49" t="n"/>
+      <c r="O60" s="49" t="n"/>
+      <c r="P60" s="50" t="n"/>
     </row>
     <row r="61" ht="80" customHeight="1">
       <c r="A61" s="41" t="inlineStr">
@@ -10698,6 +11408,20 @@
 移行時には次フェーズのTodoを「未着手」から「進行中」に更新。</t>
         </is>
       </c>
+      <c r="C61" s="49" t="n"/>
+      <c r="D61" s="49" t="n"/>
+      <c r="E61" s="49" t="n"/>
+      <c r="F61" s="49" t="n"/>
+      <c r="G61" s="49" t="n"/>
+      <c r="H61" s="49" t="n"/>
+      <c r="I61" s="49" t="n"/>
+      <c r="J61" s="49" t="n"/>
+      <c r="K61" s="49" t="n"/>
+      <c r="L61" s="49" t="n"/>
+      <c r="M61" s="49" t="n"/>
+      <c r="N61" s="49" t="n"/>
+      <c r="O61" s="49" t="n"/>
+      <c r="P61" s="50" t="n"/>
     </row>
     <row r="62" ht="80" customHeight="1">
       <c r="A62" s="41" t="inlineStr">
@@ -10711,6 +11435,20 @@
 週次レビューで優先度を判断し、Todo詳細に移動。</t>
         </is>
       </c>
+      <c r="C62" s="49" t="n"/>
+      <c r="D62" s="49" t="n"/>
+      <c r="E62" s="49" t="n"/>
+      <c r="F62" s="49" t="n"/>
+      <c r="G62" s="49" t="n"/>
+      <c r="H62" s="49" t="n"/>
+      <c r="I62" s="49" t="n"/>
+      <c r="J62" s="49" t="n"/>
+      <c r="K62" s="49" t="n"/>
+      <c r="L62" s="49" t="n"/>
+      <c r="M62" s="49" t="n"/>
+      <c r="N62" s="49" t="n"/>
+      <c r="O62" s="49" t="n"/>
+      <c r="P62" s="50" t="n"/>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="26" t="inlineStr">
@@ -10851,6 +11589,662 @@
       <c r="E70" s="28" t="inlineStr">
         <is>
           <t>→ 完了</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="48" t="inlineStr">
+        <is>
+          <t>T-47</t>
+        </is>
+      </c>
+      <c r="B72" s="48" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="C72" s="48" t="inlineStr">
+        <is>
+          <t>住宅展示場・イベント出展交渉</t>
+        </is>
+      </c>
+      <c r="D72" s="48" t="inlineStr">
+        <is>
+          <t>対面接点を増やしブランド認知向上</t>
+        </is>
+      </c>
+      <c r="E72" s="48" t="inlineStr">
+        <is>
+          <t>鹿児島の住宅展示場にぺいほーむブース出展を交渉</t>
+        </is>
+      </c>
+      <c r="F72" s="48" t="inlineStr">
+        <is>
+          <t>出展契約/ブース設計案</t>
+        </is>
+      </c>
+      <c r="G72" s="48" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="H72" s="48" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="I72" s="48" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="J72" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="K72" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L72" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M72" s="48" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N72" s="48" t="inlineStr">
+        <is>
+          <t>年2回程度のイベント出展</t>
+        </is>
+      </c>
+      <c r="O72" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P72" s="48" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="48" t="inlineStr">
+        <is>
+          <t>T-48</t>
+        </is>
+      </c>
+      <c r="B73" s="48" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="C73" s="48" t="inlineStr">
+        <is>
+          <t>火災保険・引越し業者アライアンス</t>
+        </is>
+      </c>
+      <c r="D73" s="48" t="inlineStr">
+        <is>
+          <t>周辺サービスで収益多角化</t>
+        </is>
+      </c>
+      <c r="E73" s="48" t="inlineStr">
+        <is>
+          <t>火災保険代理店/引越し業者に成約紹介料モデルを提案</t>
+        </is>
+      </c>
+      <c r="F73" s="48" t="inlineStr">
+        <is>
+          <t>アライアンス契約/紹介フロー</t>
+        </is>
+      </c>
+      <c r="G73" s="48" t="inlineStr">
+        <is>
+          <t>経営/営業</t>
+        </is>
+      </c>
+      <c r="H73" s="48" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="I73" s="48" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="J73" s="48" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="K73" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L73" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M73" s="48" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N73" s="48" t="inlineStr">
+        <is>
+          <t>成約後アフターサービス</t>
+        </is>
+      </c>
+      <c r="O73" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P73" s="48" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="48" t="inlineStr">
+        <is>
+          <t>T-49</t>
+        </is>
+      </c>
+      <c r="B74" s="48" t="inlineStr">
+        <is>
+          <t>戦略</t>
+        </is>
+      </c>
+      <c r="C74" s="48" t="inlineStr">
+        <is>
+          <t>補助金・助成金情報の定期更新</t>
+        </is>
+      </c>
+      <c r="D74" s="48" t="inlineStr">
+        <is>
+          <t>情報鮮度がプラットフォーム信頼度に直結</t>
+        </is>
+      </c>
+      <c r="E74" s="48" t="inlineStr">
+        <is>
+          <t>国/県/市の住宅関連補助金を月次で調査・更新</t>
+        </is>
+      </c>
+      <c r="F74" s="48" t="inlineStr">
+        <is>
+          <t>補助金情報一覧/更新フロー</t>
+        </is>
+      </c>
+      <c r="G74" s="48" t="inlineStr">
+        <is>
+          <t>コンテンツ</t>
+        </is>
+      </c>
+      <c r="H74" s="48" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I74" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="J74" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="K74" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L74" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M74" s="48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N74" s="48" t="inlineStr">
+        <is>
+          <t>2026年度補助金が4月発表</t>
+        </is>
+      </c>
+      <c r="O74" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P74" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="48" t="inlineStr">
+        <is>
+          <t>T-50</t>
+        </is>
+      </c>
+      <c r="B75" s="48" t="inlineStr">
+        <is>
+          <t>集客</t>
+        </is>
+      </c>
+      <c r="C75" s="48" t="inlineStr">
+        <is>
+          <t>Instagram運用開始</t>
+        </is>
+      </c>
+      <c r="D75" s="48" t="inlineStr">
+        <is>
+          <t>YouTube以外の集客チャネル確立</t>
+        </is>
+      </c>
+      <c r="E75" s="48" t="inlineStr">
+        <is>
+          <t>Instagram開設。週3投稿で平屋写真を投稿</t>
+        </is>
+      </c>
+      <c r="F75" s="48" t="inlineStr">
+        <is>
+          <t>投稿テンプレート/運用ガイド</t>
+        </is>
+      </c>
+      <c r="G75" s="48" t="inlineStr">
+        <is>
+          <t>マーケ</t>
+        </is>
+      </c>
+      <c r="H75" s="48" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="I75" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="J75" s="48" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="K75" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L75" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M75" s="48" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N75" s="48" t="inlineStr">
+        <is>
+          <t>YouTube動画カット画像を再利用</t>
+        </is>
+      </c>
+      <c r="O75" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P75" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="48" t="inlineStr">
+        <is>
+          <t>T-51</t>
+        </is>
+      </c>
+      <c r="B76" s="48" t="inlineStr">
+        <is>
+          <t>営業</t>
+        </is>
+      </c>
+      <c r="C76" s="48" t="inlineStr">
+        <is>
+          <t>既存YouTube視聴者アンケート実施</t>
+        </is>
+      </c>
+      <c r="D76" s="48" t="inlineStr">
+        <is>
+          <t>ターゲット像の解像度を上げる</t>
+        </is>
+      </c>
+      <c r="E76" s="48" t="inlineStr">
+        <is>
+          <t>YouTubeコミュニティ投稿でアンケート実施</t>
+        </is>
+      </c>
+      <c r="F76" s="48" t="inlineStr">
+        <is>
+          <t>アンケート結果/ペルソナ更新</t>
+        </is>
+      </c>
+      <c r="G76" s="48" t="inlineStr">
+        <is>
+          <t>経営/マーケ</t>
+        </is>
+      </c>
+      <c r="H76" s="48" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I76" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="J76" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="K76" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L76" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M76" s="48" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="N76" s="48" t="inlineStr">
+        <is>
+          <t>コミュニティ投稿は無料</t>
+        </is>
+      </c>
+      <c r="O76" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P76" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="48" t="inlineStr">
+        <is>
+          <t>T-52</t>
+        </is>
+      </c>
+      <c r="B77" s="48" t="inlineStr">
+        <is>
+          <t>オペ</t>
+        </is>
+      </c>
+      <c r="C77" s="48" t="inlineStr">
+        <is>
+          <t>カスタマーサポート体制構築</t>
+        </is>
+      </c>
+      <c r="D77" s="48" t="inlineStr">
+        <is>
+          <t>反響対応品質がリピート/口コミに直結</t>
+        </is>
+      </c>
+      <c r="E77" s="48" t="inlineStr">
+        <is>
+          <t>電話/メール/LINE対応の担当割り振り</t>
+        </is>
+      </c>
+      <c r="F77" s="48" t="inlineStr">
+        <is>
+          <t>対応担当表/週次シフト</t>
+        </is>
+      </c>
+      <c r="G77" s="48" t="inlineStr">
+        <is>
+          <t>経営/CS</t>
+        </is>
+      </c>
+      <c r="H77" s="48" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I77" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="J77" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="K77" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L77" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M77" s="48" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N77" s="48" t="inlineStr">
+        <is>
+          <t>オペマニュアル作成済み</t>
+        </is>
+      </c>
+      <c r="O77" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P77" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="48" t="inlineStr">
+        <is>
+          <t>T-53</t>
+        </is>
+      </c>
+      <c r="B78" s="48" t="inlineStr">
+        <is>
+          <t>品質</t>
+        </is>
+      </c>
+      <c r="C78" s="48" t="inlineStr">
+        <is>
+          <t>掲載工務店の施工事例写真収集</t>
+        </is>
+      </c>
+      <c r="D78" s="48" t="inlineStr">
+        <is>
+          <t>写真品質がCV率に直結</t>
+        </is>
+      </c>
+      <c r="E78" s="48" t="inlineStr">
+        <is>
+          <t>掲載予定工務店に施工事例写真5-10枚の提供依頼</t>
+        </is>
+      </c>
+      <c r="F78" s="48" t="inlineStr">
+        <is>
+          <t>施工事例写真セット/掲載許可書</t>
+        </is>
+      </c>
+      <c r="G78" s="48" t="inlineStr">
+        <is>
+          <t>コンテンツ/営業</t>
+        </is>
+      </c>
+      <c r="H78" s="48" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="I78" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-07</t>
+        </is>
+      </c>
+      <c r="J78" s="48" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="K78" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L78" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M78" s="48" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="N78" s="48" t="inlineStr">
+        <is>
+          <t>最低3社分確保</t>
+        </is>
+      </c>
+      <c r="O78" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P78" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="48" t="inlineStr">
+        <is>
+          <t>T-54</t>
+        </is>
+      </c>
+      <c r="B79" s="48" t="inlineStr">
+        <is>
+          <t>戦略</t>
+        </is>
+      </c>
+      <c r="C79" s="48" t="inlineStr">
+        <is>
+          <t>競合分析レポート作成</t>
+        </is>
+      </c>
+      <c r="D79" s="48" t="inlineStr">
+        <is>
+          <t>大手との差別化ポイント明確化</t>
+        </is>
+      </c>
+      <c r="E79" s="48" t="inlineStr">
+        <is>
+          <t>主要競合5サービスの機能/価格/強み/弱み整理</t>
+        </is>
+      </c>
+      <c r="F79" s="48" t="inlineStr">
+        <is>
+          <t>競合分析レポート</t>
+        </is>
+      </c>
+      <c r="G79" s="48" t="inlineStr">
+        <is>
+          <t>経営/PM</t>
+        </is>
+      </c>
+      <c r="H79" s="48" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="I79" s="48" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="J79" s="48" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="K79" s="48" t="inlineStr">
+        <is>
+          <t>未着手</t>
+        </is>
+      </c>
+      <c r="L79" s="48" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="M79" s="48" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="N79" s="48" t="inlineStr">
+        <is>
+          <t>営業提案の差別化根拠</t>
+        </is>
+      </c>
+      <c r="O79" s="48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="P79" s="48" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
         </is>
       </c>
     </row>

</xml_diff>